<commit_message>
starting edge inference script
</commit_message>
<xml_diff>
--- a/training_run_data_analysis.xlsx
+++ b/training_run_data_analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samta\programming\python\yolomg-stw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0B02D79-CBD8-4F4E-9FEF-D798B7C4DC65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4578AE66-5D6B-4A71-B838-6E5E9E47D66F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{0E0F7E5E-85CE-4CEF-BB80-A4BFDD82C860}"/>
   </bookViews>
@@ -887,9 +887,7 @@
     <col min="3" max="3" width="8.3046875" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="46" customWidth="1"/>
     <col min="5" max="5" width="13" customWidth="1"/>
-    <col min="6" max="13" width="7.765625" customWidth="1"/>
-    <col min="14" max="18" width="7.765625" hidden="1" customWidth="1"/>
-    <col min="19" max="20" width="7.765625" customWidth="1"/>
+    <col min="6" max="20" width="7.765625" customWidth="1"/>
     <col min="23" max="23" width="21.4609375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>